<commit_message>
Integrate exception queue, demo fixtures, and AO integration docs.
- Add harness/exceptions.py: detect, write, and review exception queue with evidence rows.
- Wire exceptions into harness/pipeline.py after verify; return result dict from predict_task.
- Add harness/__init__.py for `python -m harness.exceptions`.
- Fix demo fixture generation: blank answer cells correctly; add Corvus LE Reference sheet.
- Add simulate_demo.sh (offline exception queue) and run_skill_demo.sh (skill loop).
- Update run_demo.sh to use research/.venv python3 and print review command.
- Add docs/SYNDICATE-AO-INTEGRATION.md and docs/AO-SESSION-LOG.md.
- Update SYNDICATE-DEMO.md, SESSION-STATUS.md, READMEs for exception workflow and AO.

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/demo/close-tieout/spreadsheet/close-tieout-bank-cp/1_close-tieout-bank-cp_init.xlsx
+++ b/demo/close-tieout/spreadsheet/close-tieout-bank-cp/1_close-tieout-bank-cp_init.xlsx
@@ -593,11 +593,6 @@
           <t>NI ABF I SCSP</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>NI ABF I SCSp</t>
-        </is>
-      </c>
       <c r="L2" t="inlineStr">
         <is>
           <t>NI ABF I SCSp</t>
@@ -702,11 +697,6 @@
           <t>NI ABF I SCSP</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>NI ABF I SCSp</t>
-        </is>
-      </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>NI ABF I SCSp</t>
@@ -811,11 +801,6 @@
           <t>NI ABF I SCSP</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>NI ABF I SCSp</t>
-        </is>
-      </c>
       <c r="L4" t="inlineStr">
         <is>
           <t>NI ABF I SCSp</t>
@@ -989,11 +974,6 @@
           <t>NIP PLATFORM SOLUTIONS APS</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>NIP PLATFORM SOLUTIONS APS</t>
-        </is>
-      </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>NIP PLATFORM SOLUTIONS APS</t>
@@ -1076,11 +1056,6 @@
           <t>TRENTBECK AUDIT LUXEMBOURG</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Trentbeck Audit - Lu</t>
-        </is>
-      </c>
       <c r="M7" t="inlineStr">
         <is>
           <t>Vendor</t>
@@ -1165,11 +1140,6 @@
           <t>NI ABF I SCSP</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>NI ABF I SCSp</t>
-        </is>
-      </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>NI ABF I SCSp</t>
@@ -1269,11 +1239,6 @@
           <t>NI ABF I SCSP</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>NI ABF I SCSp</t>
-        </is>
-      </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>NI ABF I SCSp</t>
@@ -1378,11 +1343,6 @@
           <t>NI ABF I SCSP</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>NI ABF I SCSp</t>
-        </is>
-      </c>
       <c r="L10" t="inlineStr">
         <is>
           <t>NI ABF I SCSp</t>
@@ -1487,11 +1447,6 @@
           <t>NI ABF II MIZARCO S.A R.L.</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>NI ABF II MizarCo S.à r.l.</t>
-        </is>
-      </c>
       <c r="L11" t="inlineStr">
         <is>
           <t>NI ABF II MizarCo S.à r.l.</t>
@@ -1596,11 +1551,6 @@
           <t>NI ABF II MIZARCO S.A R.L.</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>NI ABF II MizarCo S.à r.l.</t>
-        </is>
-      </c>
       <c r="L12" t="inlineStr">
         <is>
           <t>NI ABF II MizarCo S.à r.l.</t>
@@ -1784,11 +1734,6 @@
           <t>NI ABF II MIZARCO S.A R.L.</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>NI ABF II MizarCo S.à r.l.</t>
-        </is>
-      </c>
       <c r="L14" t="inlineStr">
         <is>
           <t>NI ABF II MizarCo S.à r.l.</t>
@@ -1883,11 +1828,6 @@
           <t>ULLA B. HILLEBRANDT CONSULTING</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>Ulla B. Hillebrandt Consulting - Non-LU</t>
-        </is>
-      </c>
       <c r="M15" t="inlineStr">
         <is>
           <t>Vendor</t>
@@ -1965,11 +1905,6 @@
       <c r="J16" t="inlineStr">
         <is>
           <t>NIP LIT</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>NIP P/S</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">

</xml_diff>